<commit_message>
Docs: Update Blockdiagram with photos + Add Vermogenslijst
</commit_message>
<xml_diff>
--- a/docs/hardware/MateriaalLijst+Prijzen.xlsx
+++ b/docs/hardware/MateriaalLijst+Prijzen.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="21">
   <si>
     <t>Component</t>
   </si>
@@ -30,6 +30,9 @@
     <t>Kosten</t>
   </si>
   <si>
+    <t>Opmerkingen</t>
+  </si>
+  <si>
     <t xml:space="preserve">RasberryPi 4B (4GB RAM)</t>
   </si>
   <si>
@@ -57,10 +60,16 @@
     <t>website</t>
   </si>
   <si>
-    <t>HomeServer</t>
+    <t xml:space="preserve">HomeServe: HP EliteDesk 800 G1 SFF</t>
   </si>
   <si>
     <t xml:space="preserve">Met 2ehands materiaal</t>
+  </si>
+  <si>
+    <t>Ebay</t>
+  </si>
+  <si>
+    <t xml:space="preserve">geschatte waarde (ebay)</t>
   </si>
   <si>
     <t>Drukknop</t>
@@ -123,11 +132,10 @@
   <cellStyleXfs count="1">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
     <xf fontId="1" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1"/>
     <xf fontId="2" fillId="2" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf fontId="0" fillId="2" borderId="0" numFmtId="0" xfId="0" applyFill="1"/>
     <xf fontId="0" fillId="2" borderId="0" numFmtId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -147,13 +155,14 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" displayName="Table2" ref="$A$1:$D$10">
-  <autoFilter ref="$A$1:$D$10"/>
-  <tableColumns count="4">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" displayName="Table2" ref="A1:E10">
+  <autoFilter ref="A1:E10"/>
+  <tableColumns count="5">
     <tableColumn id="1" name="Component"/>
     <tableColumn id="2" name="Beschrijving"/>
     <tableColumn id="3" name="Link"/>
     <tableColumn id="4" name="Kosten"/>
+    <tableColumn id="5" name="Opmerkingen"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -653,10 +662,11 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="27.140625"/>
+    <col customWidth="1" min="1" max="1" width="33.28125"/>
     <col customWidth="1" min="2" max="2" width="38.57421875"/>
     <col customWidth="1" min="3" max="3" width="16.421875"/>
     <col bestFit="1" min="4" max="4" width="11.00390625"/>
+    <col customWidth="1" min="5" max="5" width="18.7109375"/>
   </cols>
   <sheetData>
     <row r="1" ht="14.25">
@@ -672,16 +682,19 @@
       <c r="D1" t="s">
         <v>3</v>
       </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
     </row>
     <row r="2" ht="14.25">
       <c r="A2" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B2" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D2">
         <v>64.120000000000005</v>
@@ -689,13 +702,13 @@
     </row>
     <row r="3" ht="14.25">
       <c r="A3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B3" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D3">
         <v>0</v>
@@ -703,13 +716,13 @@
     </row>
     <row r="4" ht="14.25">
       <c r="A4" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B4" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D4">
         <v>30</v>
@@ -717,32 +730,38 @@
     </row>
     <row r="5" ht="14.25">
       <c r="A5" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B5" t="s">
-        <v>14</v>
+        <v>15</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>16</v>
       </c>
       <c r="D5">
-        <v>0</v>
+        <v>60</v>
+      </c>
+      <c r="E5" t="s">
+        <v>17</v>
       </c>
     </row>
     <row r="6" ht="14.25">
       <c r="A6" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="B6" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
     </row>
     <row r="10" ht="14.25">
       <c r="A10" s="2" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="B10" s="3"/>
-      <c r="C10" s="4"/>
-      <c r="D10" s="4">
+      <c r="C10" s="3"/>
+      <c r="D10" s="3">
         <f>D2+D3+D4+D5+D6+D7+D8+D9</f>
-        <v>94.120000000000005</v>
+        <v>154.12</v>
       </c>
     </row>
     <row r="13" ht="14.25"/>
@@ -752,13 +771,14 @@
     <hyperlink r:id="rId1" ref="C2" tooltip=""/>
     <hyperlink r:id="rId2" ref="C3" tooltip=""/>
     <hyperlink r:id="rId3" ref="C4" tooltip=""/>
+    <hyperlink r:id="rId4" ref="C5" tooltip=""/>
   </hyperlinks>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>
   <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="0" copies="1"/>
   <headerFooter/>
   <tableParts count="1">
-    <tablePart r:id="rId4"/>
+    <tablePart r:id="rId5"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>